<commit_message>
update data after question answer
</commit_message>
<xml_diff>
--- a/Data/5G KONUMLANDIRMA YARISMA VERISI/5G Baz İstasyonu Konfigürasyon Verileri/İTÜ 5G Hücre Bilgileri.xlsx
+++ b/Data/5G KONUMLANDIRMA YARISMA VERISI/5G Baz İstasyonu Konfigürasyon Verileri/İTÜ 5G Hücre Bilgileri.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ogrharranedu-my.sharepoint.com/personal/210504131_ogrenci_harran_edu_tr/Documents/teknofest/5G-Positioning-Competition/Data/5G KONUMLANDIRMA YARISMA VERISI/5G Baz İstasyonu Konfigürasyon Verileri/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TCGKALEM\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{C188847A-A083-4C96-A701-BEA6545CEFF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C36B602-9AA2-49F8-93DF-CDD119A8AF16}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C188847A-A083-4C96-A701-BEA6545CEFF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{99887ECB-6D70-4376-A31A-BD0DC24DDF23}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{99887ECB-6D70-4376-A31A-BD0DC24DDF23}"/>
   </bookViews>
   <sheets>
     <sheet name="Hücre tablosu" sheetId="1" r:id="rId1"/>
@@ -512,8 +512,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="238125" y="390525"/>
-          <a:ext cx="5372100" cy="5052266"/>
+          <a:off x="238125" y="400050"/>
+          <a:ext cx="5372100" cy="5265626"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -571,8 +571,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="6305550" y="390527"/>
-          <a:ext cx="6162675" cy="2541268"/>
+          <a:off x="6305550" y="400052"/>
+          <a:ext cx="6162675" cy="2647948"/>
           <a:chOff x="6457950" y="342902"/>
           <a:chExt cx="5724525" cy="2295524"/>
         </a:xfrm>
@@ -697,14 +697,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Teması">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -742,7 +738,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -848,7 +844,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -990,7 +986,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -999,17 +995,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4F81FD4-A44C-4CC0-ACA4-A5CD39C48CE0}">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr defaultColWidth="15.5546875" defaultRowHeight="20.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="15.5703125" defaultRowHeight="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="15.5546875" style="9"/>
-    <col min="7" max="7" width="30.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.5546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="13" width="15.5546875" style="9"/>
-    <col min="14" max="14" width="20.88671875" style="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="15.5546875" style="9"/>
+    <col min="1" max="6" width="15.5703125" style="9"/>
+    <col min="7" max="7" width="30.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="13" width="15.5703125" style="9"/>
+    <col min="14" max="14" width="20.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="15.5703125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1053,7 +1049,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -1097,7 +1093,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -1141,7 +1137,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
@@ -1185,7 +1181,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
@@ -1229,7 +1225,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>12</v>
       </c>
@@ -1273,7 +1269,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
@@ -1317,7 +1313,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
@@ -1361,7 +1357,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
@@ -1405,7 +1401,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>16</v>
       </c>
@@ -1461,9 +1457,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{949C38FA-3220-4727-AA8F-D54EB4755E2F}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>31</v>
       </c>

</xml_diff>